<commit_message>
update test cases and algorithm
</commit_message>
<xml_diff>
--- a/test/config/case20/ring_case.xlsx
+++ b/test/config/case20/ring_case.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255" firstSheet="2" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="10455" firstSheet="2" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="muyan信号与bumpbank对应关系" sheetId="2" r:id="rId1"/>
@@ -5187,8 +5187,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8413115" y="6383655"/>
-          <a:ext cx="10832465" cy="4645660"/>
+          <a:off x="8413115" y="6322695"/>
+          <a:ext cx="10832465" cy="4528820"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5230,7 +5230,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="31750" y="285115"/>
-          <a:ext cx="7410450" cy="5260975"/>
+          <a:ext cx="7410450" cy="5225415"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5272,7 +5272,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8291830" y="358775"/>
-          <a:ext cx="10610850" cy="5244465"/>
+          <a:ext cx="10610850" cy="5208905"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6646,7 +6646,7 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:13">
-      <c r="A2" s="13">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="15" t="s">
@@ -6674,8 +6674,7 @@
       <c r="L2" s="40"/>
       <c r="M2" s="41"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:13">
-      <c r="A3" s="13"/>
+    <row r="3" ht="15" customHeight="1" spans="2:13">
       <c r="B3" s="18" t="s">
         <v>249</v>
       </c>
@@ -6697,8 +6696,7 @@
       <c r="L3" s="43"/>
       <c r="M3" s="44"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:13">
-      <c r="A4" s="13"/>
+    <row r="4" ht="15" customHeight="1" spans="2:13">
       <c r="B4" s="18" t="s">
         <v>251</v>
       </c>
@@ -6720,8 +6718,7 @@
       <c r="L4" s="43"/>
       <c r="M4" s="44"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:13">
-      <c r="A5" s="13"/>
+    <row r="5" ht="15" customHeight="1" spans="2:13">
       <c r="B5" s="21" t="s">
         <v>253</v>
       </c>
@@ -6743,8 +6740,7 @@
       <c r="L5" s="43"/>
       <c r="M5" s="44"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:13">
-      <c r="A6" s="13"/>
+    <row r="6" ht="15" customHeight="1" spans="2:13">
       <c r="B6" s="24" t="s">
         <v>255</v>
       </c>
@@ -6766,8 +6762,7 @@
       <c r="L6" s="43"/>
       <c r="M6" s="44"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:13">
-      <c r="A7" s="13"/>
+    <row r="7" ht="15" customHeight="1" spans="2:13">
       <c r="B7" s="28" t="s">
         <v>257</v>
       </c>
@@ -6789,8 +6784,7 @@
       <c r="L7" s="43"/>
       <c r="M7" s="44"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:13">
-      <c r="A8" s="13"/>
+    <row r="8" ht="15" customHeight="1" spans="2:13">
       <c r="B8" s="28" t="s">
         <v>259</v>
       </c>
@@ -6812,8 +6806,7 @@
       <c r="L8" s="43"/>
       <c r="M8" s="44"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:13">
-      <c r="A9" s="13"/>
+    <row r="9" ht="15" customHeight="1" spans="2:13">
       <c r="B9" s="28" t="s">
         <v>261</v>
       </c>
@@ -6835,8 +6828,7 @@
       <c r="L9" s="46"/>
       <c r="M9" s="47"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:9">
-      <c r="A10" s="13"/>
+    <row r="10" ht="15" customHeight="1" spans="2:9">
       <c r="B10" s="28" t="s">
         <v>263</v>
       </c>
@@ -6855,8 +6847,7 @@
       </c>
       <c r="I10" s="29"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:9">
-      <c r="A11" s="13"/>
+    <row r="11" ht="15" customHeight="1" spans="2:9">
       <c r="B11" s="28" t="s">
         <v>265</v>
       </c>
@@ -6875,8 +6866,7 @@
       </c>
       <c r="I11" s="29"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:9">
-      <c r="A12" s="13"/>
+    <row r="12" ht="15" customHeight="1" spans="2:9">
       <c r="B12" s="28" t="s">
         <v>267</v>
       </c>
@@ -6895,8 +6885,7 @@
       </c>
       <c r="I12" s="29"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:9">
-      <c r="A13" s="13"/>
+    <row r="13" ht="15" customHeight="1" spans="2:9">
       <c r="B13" s="28" t="s">
         <v>269</v>
       </c>
@@ -6915,8 +6904,7 @@
       </c>
       <c r="I13" s="29"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:9">
-      <c r="A14" s="13"/>
+    <row r="14" ht="15" customHeight="1" spans="2:9">
       <c r="B14" s="28" t="s">
         <v>271</v>
       </c>
@@ -6935,8 +6923,7 @@
       </c>
       <c r="I14" s="29"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:9">
-      <c r="A15" s="13"/>
+    <row r="15" ht="15" customHeight="1" spans="2:9">
       <c r="B15" s="28" t="s">
         <v>273</v>
       </c>
@@ -6955,8 +6942,7 @@
       </c>
       <c r="I15" s="29"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:9">
-      <c r="A16" s="13"/>
+    <row r="16" ht="15" customHeight="1" spans="2:9">
       <c r="B16" s="28" t="s">
         <v>275</v>
       </c>
@@ -6975,8 +6961,7 @@
       </c>
       <c r="I16" s="29"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:9">
-      <c r="A17" s="13"/>
+    <row r="17" ht="15" customHeight="1" spans="2:9">
       <c r="B17" s="30" t="s">
         <v>277</v>
       </c>
@@ -6995,8 +6980,7 @@
       </c>
       <c r="I17" s="32"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:9">
-      <c r="A18" s="13"/>
+    <row r="18" ht="15" customHeight="1" spans="2:9">
       <c r="B18" s="33" t="s">
         <v>279</v>
       </c>
@@ -7015,8 +6999,7 @@
       </c>
       <c r="I18" s="35"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:9">
-      <c r="A19" s="13"/>
+    <row r="19" ht="15" customHeight="1" spans="2:9">
       <c r="B19" s="28" t="s">
         <v>281</v>
       </c>
@@ -7035,8 +7018,7 @@
       </c>
       <c r="I19" s="29"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:9">
-      <c r="A20" s="13"/>
+    <row r="20" ht="15" customHeight="1" spans="2:9">
       <c r="B20" s="28" t="s">
         <v>283</v>
       </c>
@@ -7055,8 +7037,7 @@
       </c>
       <c r="I20" s="29"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:9">
-      <c r="A21" s="13"/>
+    <row r="21" ht="15" customHeight="1" spans="2:9">
       <c r="B21" s="28" t="s">
         <v>285</v>
       </c>
@@ -7075,8 +7056,7 @@
       </c>
       <c r="I21" s="29"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:9">
-      <c r="A22" s="13"/>
+    <row r="22" ht="15" customHeight="1" spans="2:9">
       <c r="B22" s="28" t="s">
         <v>287</v>
       </c>
@@ -7095,8 +7075,7 @@
       </c>
       <c r="I22" s="29"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:9">
-      <c r="A23" s="13"/>
+    <row r="23" ht="15" customHeight="1" spans="2:9">
       <c r="B23" s="28" t="s">
         <v>289</v>
       </c>
@@ -7115,8 +7094,7 @@
       </c>
       <c r="I23" s="29"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:9">
-      <c r="A24" s="13"/>
+    <row r="24" ht="15" customHeight="1" spans="2:9">
       <c r="B24" s="28" t="s">
         <v>291</v>
       </c>
@@ -7135,8 +7113,7 @@
       </c>
       <c r="I24" s="29"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:9">
-      <c r="A25" s="13"/>
+    <row r="25" ht="15" customHeight="1" spans="2:9">
       <c r="B25" s="28" t="s">
         <v>293</v>
       </c>
@@ -7155,8 +7132,7 @@
       </c>
       <c r="I25" s="29"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:9">
-      <c r="A26" s="13"/>
+    <row r="26" ht="15" customHeight="1" spans="2:9">
       <c r="B26" s="28" t="s">
         <v>295</v>
       </c>
@@ -7175,8 +7151,7 @@
       </c>
       <c r="I26" s="29"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:9">
-      <c r="A27" s="13"/>
+    <row r="27" ht="15" customHeight="1" spans="2:9">
       <c r="B27" s="28" t="s">
         <v>297</v>
       </c>
@@ -7195,8 +7170,7 @@
       </c>
       <c r="I27" s="29"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:9">
-      <c r="A28" s="13"/>
+    <row r="28" ht="15" customHeight="1" spans="2:9">
       <c r="B28" s="28" t="s">
         <v>299</v>
       </c>
@@ -7215,8 +7189,7 @@
       </c>
       <c r="I28" s="29"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:9">
-      <c r="A29" s="13"/>
+    <row r="29" ht="15" customHeight="1" spans="2:9">
       <c r="B29" s="28" t="s">
         <v>301</v>
       </c>
@@ -7235,8 +7208,7 @@
       </c>
       <c r="I29" s="29"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:9">
-      <c r="A30" s="13"/>
+    <row r="30" ht="15" customHeight="1" spans="2:9">
       <c r="B30" s="28" t="s">
         <v>303</v>
       </c>
@@ -7255,8 +7227,7 @@
       </c>
       <c r="I30" s="29"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:9">
-      <c r="A31" s="13"/>
+    <row r="31" ht="15" customHeight="1" spans="2:9">
       <c r="B31" s="28" t="s">
         <v>305</v>
       </c>
@@ -7275,8 +7246,7 @@
       </c>
       <c r="I31" s="29"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:9">
-      <c r="A32" s="13"/>
+    <row r="32" ht="15" customHeight="1" spans="2:9">
       <c r="B32" s="28" t="s">
         <v>307</v>
       </c>
@@ -7295,8 +7265,7 @@
       </c>
       <c r="I32" s="29"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:9">
-      <c r="A33" s="13"/>
+    <row r="33" ht="15" customHeight="1" spans="2:9">
       <c r="B33" s="28" t="s">
         <v>309</v>
       </c>
@@ -7315,8 +7284,7 @@
       </c>
       <c r="I33" s="29"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:9">
-      <c r="A34" s="13"/>
+    <row r="34" ht="15" customHeight="1" spans="2:9">
       <c r="B34" s="28" t="s">
         <v>311</v>
       </c>
@@ -7335,8 +7303,7 @@
       </c>
       <c r="I34" s="29"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:9">
-      <c r="A35" s="13"/>
+    <row r="35" ht="15" customHeight="1" spans="2:9">
       <c r="B35" s="28" t="s">
         <v>313</v>
       </c>
@@ -7355,8 +7322,7 @@
       </c>
       <c r="I35" s="29"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:9">
-      <c r="A36" s="13"/>
+    <row r="36" ht="15" customHeight="1" spans="2:9">
       <c r="B36" s="28" t="s">
         <v>315</v>
       </c>
@@ -7375,8 +7341,7 @@
       </c>
       <c r="I36" s="29"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:9">
-      <c r="A37" s="13"/>
+    <row r="37" ht="15" customHeight="1" spans="2:9">
       <c r="B37" s="36" t="s">
         <v>317</v>
       </c>
@@ -7395,8 +7360,7 @@
       </c>
       <c r="I37" s="38"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:9">
-      <c r="A38" s="13"/>
+    <row r="38" ht="15" customHeight="1" spans="2:9">
       <c r="B38" s="24" t="s">
         <v>319</v>
       </c>
@@ -7413,8 +7377,7 @@
       </c>
       <c r="I38" s="26"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:9">
-      <c r="A39" s="13"/>
+    <row r="39" ht="15" customHeight="1" spans="2:9">
       <c r="B39" s="28" t="s">
         <v>322</v>
       </c>
@@ -7431,8 +7394,7 @@
       </c>
       <c r="I39" s="29"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:9">
-      <c r="A40" s="13"/>
+    <row r="40" ht="15" customHeight="1" spans="2:9">
       <c r="B40" s="28" t="s">
         <v>325</v>
       </c>
@@ -7449,8 +7411,7 @@
       </c>
       <c r="I40" s="29"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:9">
-      <c r="A41" s="13"/>
+    <row r="41" ht="15" customHeight="1" spans="2:9">
       <c r="B41" s="28" t="s">
         <v>328</v>
       </c>
@@ -7467,8 +7428,7 @@
       </c>
       <c r="I41" s="29"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:9">
-      <c r="A42" s="13"/>
+    <row r="42" ht="15" customHeight="1" spans="2:9">
       <c r="B42" s="28" t="s">
         <v>331</v>
       </c>
@@ -7485,8 +7445,7 @@
       </c>
       <c r="I42" s="29"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:9">
-      <c r="A43" s="13"/>
+    <row r="43" ht="15" customHeight="1" spans="2:9">
       <c r="B43" s="28" t="s">
         <v>334</v>
       </c>
@@ -7503,8 +7462,7 @@
       </c>
       <c r="I43" s="29"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:9">
-      <c r="A44" s="13"/>
+    <row r="44" ht="15" customHeight="1" spans="2:9">
       <c r="B44" s="28" t="s">
         <v>337</v>
       </c>
@@ -7521,8 +7479,7 @@
       </c>
       <c r="I44" s="29"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:9">
-      <c r="A45" s="13"/>
+    <row r="45" ht="15" customHeight="1" spans="2:9">
       <c r="B45" s="28" t="s">
         <v>340</v>
       </c>
@@ -7539,8 +7496,7 @@
       </c>
       <c r="I45" s="29"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:9">
-      <c r="A46" s="13"/>
+    <row r="46" ht="15" customHeight="1" spans="2:9">
       <c r="B46" s="28" t="s">
         <v>343</v>
       </c>
@@ -7557,8 +7513,7 @@
       </c>
       <c r="I46" s="29"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:9">
-      <c r="A47" s="13"/>
+    <row r="47" ht="15" customHeight="1" spans="2:9">
       <c r="B47" s="28" t="s">
         <v>346</v>
       </c>
@@ -7575,8 +7530,7 @@
       </c>
       <c r="I47" s="29"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:9">
-      <c r="A48" s="13"/>
+    <row r="48" ht="15" customHeight="1" spans="2:9">
       <c r="B48" s="28" t="s">
         <v>349</v>
       </c>
@@ -7593,8 +7547,7 @@
       </c>
       <c r="I48" s="29"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:9">
-      <c r="A49" s="13"/>
+    <row r="49" ht="15" customHeight="1" spans="2:9">
       <c r="B49" s="30" t="s">
         <v>352</v>
       </c>
@@ -7611,8 +7564,7 @@
       </c>
       <c r="I49" s="32"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:9">
-      <c r="A50" s="13"/>
+    <row r="50" ht="15" customHeight="1" spans="2:9">
       <c r="B50" s="33" t="s">
         <v>355</v>
       </c>
@@ -7629,8 +7581,7 @@
       </c>
       <c r="I50" s="35"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:9">
-      <c r="A51" s="13"/>
+    <row r="51" ht="15" customHeight="1" spans="2:9">
       <c r="B51" s="28" t="s">
         <v>358</v>
       </c>
@@ -7647,8 +7598,7 @@
       </c>
       <c r="I51" s="29"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:9">
-      <c r="A52" s="13"/>
+    <row r="52" ht="15" customHeight="1" spans="2:9">
       <c r="B52" s="28" t="s">
         <v>361</v>
       </c>
@@ -7665,8 +7615,7 @@
       </c>
       <c r="I52" s="29"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:9">
-      <c r="A53" s="13"/>
+    <row r="53" ht="15" customHeight="1" spans="2:9">
       <c r="B53" s="28" t="s">
         <v>364</v>
       </c>
@@ -7683,8 +7632,7 @@
       </c>
       <c r="I53" s="29"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:9">
-      <c r="A54" s="13"/>
+    <row r="54" ht="15" customHeight="1" spans="2:9">
       <c r="B54" s="28" t="s">
         <v>367</v>
       </c>
@@ -7701,8 +7649,7 @@
       </c>
       <c r="I54" s="29"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:9">
-      <c r="A55" s="13"/>
+    <row r="55" ht="15" customHeight="1" spans="2:9">
       <c r="B55" s="28" t="s">
         <v>370</v>
       </c>
@@ -7719,8 +7666,7 @@
       </c>
       <c r="I55" s="29"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:9">
-      <c r="A56" s="13"/>
+    <row r="56" ht="15" customHeight="1" spans="2:9">
       <c r="B56" s="28" t="s">
         <v>373</v>
       </c>
@@ -7737,8 +7683,7 @@
       </c>
       <c r="I56" s="29"/>
     </row>
-    <row r="57" ht="15" customHeight="1" spans="1:9">
-      <c r="A57" s="13"/>
+    <row r="57" ht="15" customHeight="1" spans="2:9">
       <c r="B57" s="28" t="s">
         <v>376</v>
       </c>
@@ -7755,8 +7700,7 @@
       </c>
       <c r="I57" s="29"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:9">
-      <c r="A58" s="13"/>
+    <row r="58" ht="15" customHeight="1" spans="2:9">
       <c r="B58" s="28" t="s">
         <v>379</v>
       </c>
@@ -7772,8 +7716,7 @@
       </c>
       <c r="I58" s="29"/>
     </row>
-    <row r="59" ht="15" customHeight="1" spans="1:9">
-      <c r="A59" s="13"/>
+    <row r="59" ht="15" customHeight="1" spans="2:9">
       <c r="B59" s="28" t="s">
         <v>382</v>
       </c>
@@ -7789,8 +7732,7 @@
       </c>
       <c r="I59" s="29"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:9">
-      <c r="A60" s="13"/>
+    <row r="60" ht="15" customHeight="1" spans="2:9">
       <c r="B60" s="28" t="s">
         <v>385</v>
       </c>
@@ -7806,8 +7748,7 @@
       </c>
       <c r="I60" s="29"/>
     </row>
-    <row r="61" ht="15" customHeight="1" spans="1:9">
-      <c r="A61" s="13"/>
+    <row r="61" ht="15" customHeight="1" spans="2:9">
       <c r="B61" s="28" t="s">
         <v>388</v>
       </c>
@@ -7823,8 +7764,7 @@
       </c>
       <c r="I61" s="29"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:9">
-      <c r="A62" s="13"/>
+    <row r="62" ht="15" customHeight="1" spans="2:9">
       <c r="B62" s="28" t="s">
         <v>391</v>
       </c>
@@ -7840,8 +7780,7 @@
       </c>
       <c r="I62" s="29"/>
     </row>
-    <row r="63" ht="15" customHeight="1" spans="1:9">
-      <c r="A63" s="13"/>
+    <row r="63" ht="15" customHeight="1" spans="2:9">
       <c r="B63" s="28" t="s">
         <v>394</v>
       </c>
@@ -7857,8 +7796,7 @@
       </c>
       <c r="I63" s="29"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:9">
-      <c r="A64" s="13"/>
+    <row r="64" ht="15" customHeight="1" spans="2:9">
       <c r="B64" s="28" t="s">
         <v>397</v>
       </c>
@@ -7874,8 +7812,7 @@
       </c>
       <c r="I64" s="29"/>
     </row>
-    <row r="65" ht="15" customHeight="1" spans="1:9">
-      <c r="A65" s="13"/>
+    <row r="65" ht="15" customHeight="1" spans="2:9">
       <c r="B65" s="28" t="s">
         <v>400</v>
       </c>
@@ -7891,8 +7828,7 @@
       </c>
       <c r="I65" s="29"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:9">
-      <c r="A66" s="13"/>
+    <row r="66" ht="15" customHeight="1" spans="2:9">
       <c r="B66" s="28" t="s">
         <v>403</v>
       </c>
@@ -7908,8 +7844,7 @@
       </c>
       <c r="I66" s="29"/>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:9">
-      <c r="A67" s="13"/>
+    <row r="67" ht="15" customHeight="1" spans="2:9">
       <c r="B67" s="28" t="s">
         <v>406</v>
       </c>
@@ -7925,8 +7860,7 @@
       </c>
       <c r="I67" s="29"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:9">
-      <c r="A68" s="13"/>
+    <row r="68" ht="15" customHeight="1" spans="2:9">
       <c r="B68" s="28" t="s">
         <v>409</v>
       </c>
@@ -7942,8 +7876,7 @@
       </c>
       <c r="I68" s="29"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:9">
-      <c r="A69" s="13"/>
+    <row r="69" ht="15" customHeight="1" spans="2:9">
       <c r="B69" s="36" t="s">
         <v>412</v>
       </c>
@@ -7959,8 +7892,7 @@
       </c>
       <c r="I69" s="38"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:9">
-      <c r="A70" s="13"/>
+    <row r="70" ht="15" customHeight="1" spans="2:9">
       <c r="B70" s="24" t="s">
         <v>415</v>
       </c>
@@ -7976,8 +7908,7 @@
       </c>
       <c r="I70" s="26"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:9">
-      <c r="A71" s="13"/>
+    <row r="71" ht="15" customHeight="1" spans="2:9">
       <c r="B71" s="28" t="s">
         <v>419</v>
       </c>
@@ -7993,8 +7924,7 @@
       </c>
       <c r="I71" s="29"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:9">
-      <c r="A72" s="13"/>
+    <row r="72" ht="15" customHeight="1" spans="2:9">
       <c r="B72" s="28" t="s">
         <v>423</v>
       </c>
@@ -8010,8 +7940,7 @@
       </c>
       <c r="I72" s="29"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:9">
-      <c r="A73" s="13"/>
+    <row r="73" ht="15" customHeight="1" spans="2:9">
       <c r="B73" s="28" t="s">
         <v>427</v>
       </c>
@@ -8027,8 +7956,7 @@
       </c>
       <c r="I73" s="29"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:9">
-      <c r="A74" s="13"/>
+    <row r="74" ht="15" customHeight="1" spans="2:9">
       <c r="B74" s="28" t="s">
         <v>431</v>
       </c>
@@ -8044,8 +7972,7 @@
       </c>
       <c r="I74" s="29"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:9">
-      <c r="A75" s="13"/>
+    <row r="75" ht="15" customHeight="1" spans="2:9">
       <c r="B75" s="28" t="s">
         <v>435</v>
       </c>
@@ -8061,8 +7988,7 @@
       </c>
       <c r="I75" s="29"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:9">
-      <c r="A76" s="13"/>
+    <row r="76" ht="15" customHeight="1" spans="2:9">
       <c r="B76" s="28" t="s">
         <v>439</v>
       </c>
@@ -8078,8 +8004,7 @@
       </c>
       <c r="I76" s="29"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:9">
-      <c r="A77" s="13"/>
+    <row r="77" ht="15" customHeight="1" spans="2:9">
       <c r="B77" s="28" t="s">
         <v>443</v>
       </c>
@@ -8095,8 +8020,7 @@
       </c>
       <c r="I77" s="29"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:9">
-      <c r="A78" s="13"/>
+    <row r="78" ht="15" customHeight="1" spans="2:9">
       <c r="B78" s="28" t="s">
         <v>447</v>
       </c>
@@ -8112,8 +8036,7 @@
       </c>
       <c r="I78" s="29"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:9">
-      <c r="A79" s="13"/>
+    <row r="79" ht="15" customHeight="1" spans="2:9">
       <c r="B79" s="28" t="s">
         <v>451</v>
       </c>
@@ -8129,8 +8052,7 @@
       </c>
       <c r="I79" s="29"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:9">
-      <c r="A80" s="13"/>
+    <row r="80" ht="15" customHeight="1" spans="2:9">
       <c r="B80" s="28" t="s">
         <v>455</v>
       </c>
@@ -8146,8 +8068,7 @@
       </c>
       <c r="I80" s="29"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:9">
-      <c r="A81" s="13"/>
+    <row r="81" ht="15" customHeight="1" spans="2:9">
       <c r="B81" s="30" t="s">
         <v>459</v>
       </c>
@@ -8163,8 +8084,7 @@
       </c>
       <c r="I81" s="32"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:9">
-      <c r="A82" s="13"/>
+    <row r="82" ht="15" customHeight="1" spans="2:9">
       <c r="B82" s="33" t="s">
         <v>463</v>
       </c>
@@ -8180,8 +8100,7 @@
       </c>
       <c r="I82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:9">
-      <c r="A83" s="13"/>
+    <row r="83" ht="15" customHeight="1" spans="2:9">
       <c r="B83" s="28" t="s">
         <v>467</v>
       </c>
@@ -8197,8 +8116,7 @@
       </c>
       <c r="I83" s="29"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:9">
-      <c r="A84" s="13"/>
+    <row r="84" ht="15" customHeight="1" spans="2:9">
       <c r="B84" s="28" t="s">
         <v>471</v>
       </c>
@@ -8214,8 +8132,7 @@
       </c>
       <c r="I84" s="29"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:9">
-      <c r="A85" s="13"/>
+    <row r="85" ht="15" customHeight="1" spans="2:9">
       <c r="B85" s="28" t="s">
         <v>475</v>
       </c>
@@ -8231,8 +8148,7 @@
       </c>
       <c r="I85" s="29"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:9">
-      <c r="A86" s="13"/>
+    <row r="86" ht="15" customHeight="1" spans="2:9">
       <c r="B86" s="28" t="s">
         <v>479</v>
       </c>
@@ -8248,8 +8164,7 @@
       </c>
       <c r="I86" s="29"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:9">
-      <c r="A87" s="13"/>
+    <row r="87" ht="15" customHeight="1" spans="2:9">
       <c r="B87" s="28" t="s">
         <v>483</v>
       </c>
@@ -8265,8 +8180,7 @@
       </c>
       <c r="I87" s="29"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:9">
-      <c r="A88" s="13"/>
+    <row r="88" ht="15" customHeight="1" spans="2:9">
       <c r="B88" s="28" t="s">
         <v>487</v>
       </c>
@@ -8282,8 +8196,7 @@
       </c>
       <c r="I88" s="29"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:9">
-      <c r="A89" s="13"/>
+    <row r="89" ht="15" customHeight="1" spans="2:9">
       <c r="B89" s="28" t="s">
         <v>491</v>
       </c>
@@ -8299,8 +8212,7 @@
       </c>
       <c r="I89" s="29"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:9">
-      <c r="A90" s="13"/>
+    <row r="90" ht="15" customHeight="1" spans="2:9">
       <c r="B90" s="28" t="s">
         <v>495</v>
       </c>
@@ -8316,8 +8228,7 @@
       </c>
       <c r="I90" s="29"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:9">
-      <c r="A91" s="13"/>
+    <row r="91" ht="15" customHeight="1" spans="2:9">
       <c r="B91" s="28" t="s">
         <v>499</v>
       </c>
@@ -8333,8 +8244,7 @@
       </c>
       <c r="I91" s="29"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:9">
-      <c r="A92" s="13"/>
+    <row r="92" ht="15" customHeight="1" spans="2:9">
       <c r="B92" s="28" t="s">
         <v>503</v>
       </c>
@@ -8350,8 +8260,7 @@
       </c>
       <c r="I92" s="29"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:9">
-      <c r="A93" s="13"/>
+    <row r="93" ht="15" customHeight="1" spans="2:9">
       <c r="B93" s="28" t="s">
         <v>507</v>
       </c>
@@ -8367,8 +8276,7 @@
       </c>
       <c r="I93" s="29"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:9">
-      <c r="A94" s="13"/>
+    <row r="94" ht="15" customHeight="1" spans="2:9">
       <c r="B94" s="28" t="s">
         <v>511</v>
       </c>
@@ -8384,8 +8292,7 @@
       </c>
       <c r="I94" s="29"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:9">
-      <c r="A95" s="13"/>
+    <row r="95" ht="15" customHeight="1" spans="2:9">
       <c r="B95" s="28" t="s">
         <v>515</v>
       </c>
@@ -8401,8 +8308,7 @@
       </c>
       <c r="I95" s="29"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:9">
-      <c r="A96" s="13"/>
+    <row r="96" ht="15" customHeight="1" spans="2:9">
       <c r="B96" s="28" t="s">
         <v>519</v>
       </c>
@@ -8418,8 +8324,7 @@
       </c>
       <c r="I96" s="29"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:9">
-      <c r="A97" s="13"/>
+    <row r="97" ht="15" customHeight="1" spans="2:9">
       <c r="B97" s="28" t="s">
         <v>523</v>
       </c>
@@ -8435,8 +8340,7 @@
       </c>
       <c r="I97" s="29"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:9">
-      <c r="A98" s="13"/>
+    <row r="98" ht="15" customHeight="1" spans="2:9">
       <c r="B98" s="28" t="s">
         <v>527</v>
       </c>
@@ -8452,8 +8356,7 @@
       </c>
       <c r="I98" s="29"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:9">
-      <c r="A99" s="13"/>
+    <row r="99" ht="15" customHeight="1" spans="2:9">
       <c r="B99" s="28" t="s">
         <v>531</v>
       </c>
@@ -8469,8 +8372,7 @@
       </c>
       <c r="I99" s="29"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:9">
-      <c r="A100" s="13"/>
+    <row r="100" ht="15" customHeight="1" spans="2:9">
       <c r="B100" s="28" t="s">
         <v>535</v>
       </c>
@@ -8486,8 +8388,7 @@
       </c>
       <c r="I100" s="29"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:9">
-      <c r="A101" s="13"/>
+    <row r="101" ht="15" customHeight="1" spans="2:9">
       <c r="B101" s="36" t="s">
         <v>539</v>
       </c>
@@ -8503,8 +8404,7 @@
       </c>
       <c r="I101" s="38"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:9">
-      <c r="A102" s="13"/>
+    <row r="102" ht="15" customHeight="1" spans="2:9">
       <c r="B102" s="24" t="s">
         <v>543</v>
       </c>
@@ -8520,8 +8420,7 @@
       </c>
       <c r="I102" s="26"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:9">
-      <c r="A103" s="13"/>
+    <row r="103" ht="15" customHeight="1" spans="2:9">
       <c r="B103" s="28" t="s">
         <v>547</v>
       </c>
@@ -8537,8 +8436,7 @@
       </c>
       <c r="I103" s="29"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:9">
-      <c r="A104" s="13"/>
+    <row r="104" ht="15" customHeight="1" spans="2:9">
       <c r="B104" s="28" t="s">
         <v>551</v>
       </c>
@@ -8554,8 +8452,7 @@
       </c>
       <c r="I104" s="29"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:9">
-      <c r="A105" s="13"/>
+    <row r="105" ht="15" customHeight="1" spans="2:9">
       <c r="B105" s="28" t="s">
         <v>555</v>
       </c>
@@ -8571,8 +8468,7 @@
       </c>
       <c r="I105" s="29"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:9">
-      <c r="A106" s="13"/>
+    <row r="106" ht="15" customHeight="1" spans="2:9">
       <c r="B106" s="28" t="s">
         <v>559</v>
       </c>
@@ -8588,8 +8484,7 @@
       </c>
       <c r="I106" s="29"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:9">
-      <c r="A107" s="13"/>
+    <row r="107" ht="15" customHeight="1" spans="2:9">
       <c r="B107" s="28" t="s">
         <v>563</v>
       </c>
@@ -8605,8 +8500,7 @@
       </c>
       <c r="I107" s="29"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:9">
-      <c r="A108" s="13"/>
+    <row r="108" ht="15" customHeight="1" spans="2:9">
       <c r="B108" s="28" t="s">
         <v>567</v>
       </c>
@@ -8622,8 +8516,7 @@
       </c>
       <c r="I108" s="29"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:9">
-      <c r="A109" s="13"/>
+    <row r="109" ht="15" customHeight="1" spans="2:9">
       <c r="B109" s="28" t="s">
         <v>571</v>
       </c>
@@ -8639,8 +8532,7 @@
       </c>
       <c r="I109" s="29"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:9">
-      <c r="A110" s="13"/>
+    <row r="110" ht="15" customHeight="1" spans="2:9">
       <c r="B110" s="28" t="s">
         <v>575</v>
       </c>
@@ -8656,8 +8548,7 @@
       </c>
       <c r="I110" s="29"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:9">
-      <c r="A111" s="13"/>
+    <row r="111" ht="15" customHeight="1" spans="2:9">
       <c r="B111" s="28" t="s">
         <v>579</v>
       </c>
@@ -8673,8 +8564,7 @@
       </c>
       <c r="I111" s="29"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:9">
-      <c r="A112" s="13"/>
+    <row r="112" ht="15" customHeight="1" spans="2:9">
       <c r="B112" s="28" t="s">
         <v>583</v>
       </c>
@@ -8690,8 +8580,7 @@
       </c>
       <c r="I112" s="29"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:9">
-      <c r="A113" s="13"/>
+    <row r="113" ht="15" customHeight="1" spans="2:9">
       <c r="B113" s="30" t="s">
         <v>587</v>
       </c>
@@ -8707,8 +8596,7 @@
       </c>
       <c r="I113" s="32"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:9">
-      <c r="A114" s="13"/>
+    <row r="114" ht="15" customHeight="1" spans="2:9">
       <c r="B114" s="33" t="s">
         <v>591</v>
       </c>
@@ -8724,8 +8612,7 @@
       </c>
       <c r="I114" s="35"/>
     </row>
-    <row r="115" ht="15" customHeight="1" spans="1:9">
-      <c r="A115" s="13"/>
+    <row r="115" ht="15" customHeight="1" spans="2:9">
       <c r="B115" s="28" t="s">
         <v>595</v>
       </c>
@@ -8741,8 +8628,7 @@
       </c>
       <c r="I115" s="29"/>
     </row>
-    <row r="116" ht="15" customHeight="1" spans="1:9">
-      <c r="A116" s="13"/>
+    <row r="116" ht="15" customHeight="1" spans="2:9">
       <c r="B116" s="28" t="s">
         <v>599</v>
       </c>
@@ -8758,8 +8644,7 @@
       </c>
       <c r="I116" s="29"/>
     </row>
-    <row r="117" ht="15" customHeight="1" spans="1:9">
-      <c r="A117" s="13"/>
+    <row r="117" ht="15" customHeight="1" spans="2:9">
       <c r="B117" s="28" t="s">
         <v>603</v>
       </c>
@@ -8775,8 +8660,7 @@
       </c>
       <c r="I117" s="29"/>
     </row>
-    <row r="118" ht="15" customHeight="1" spans="1:9">
-      <c r="A118" s="13"/>
+    <row r="118" ht="15" customHeight="1" spans="2:9">
       <c r="B118" s="28" t="s">
         <v>607</v>
       </c>
@@ -8792,8 +8676,7 @@
       </c>
       <c r="I118" s="29"/>
     </row>
-    <row r="119" ht="15" customHeight="1" spans="1:9">
-      <c r="A119" s="13"/>
+    <row r="119" ht="15" customHeight="1" spans="2:9">
       <c r="B119" s="28" t="s">
         <v>611</v>
       </c>
@@ -8809,8 +8692,7 @@
       </c>
       <c r="I119" s="29"/>
     </row>
-    <row r="120" ht="15" customHeight="1" spans="1:9">
-      <c r="A120" s="13"/>
+    <row r="120" ht="15" customHeight="1" spans="2:9">
       <c r="B120" s="28" t="s">
         <v>615</v>
       </c>
@@ -8826,8 +8708,7 @@
       </c>
       <c r="I120" s="29"/>
     </row>
-    <row r="121" ht="15" customHeight="1" spans="1:9">
-      <c r="A121" s="13"/>
+    <row r="121" ht="15" customHeight="1" spans="2:9">
       <c r="B121" s="28" t="s">
         <v>619</v>
       </c>
@@ -8843,8 +8724,7 @@
       </c>
       <c r="I121" s="29"/>
     </row>
-    <row r="122" ht="15" customHeight="1" spans="1:9">
-      <c r="A122" s="13"/>
+    <row r="122" ht="15" customHeight="1" spans="2:9">
       <c r="B122" s="28" t="s">
         <v>623</v>
       </c>
@@ -8860,8 +8740,7 @@
       </c>
       <c r="I122" s="29"/>
     </row>
-    <row r="123" ht="15" customHeight="1" spans="1:9">
-      <c r="A123" s="13"/>
+    <row r="123" ht="15" customHeight="1" spans="2:9">
       <c r="B123" s="28" t="s">
         <v>627</v>
       </c>
@@ -8877,8 +8756,7 @@
       </c>
       <c r="I123" s="29"/>
     </row>
-    <row r="124" ht="15" customHeight="1" spans="1:9">
-      <c r="A124" s="13"/>
+    <row r="124" ht="15" customHeight="1" spans="2:9">
       <c r="B124" s="28" t="s">
         <v>631</v>
       </c>
@@ -8894,8 +8772,7 @@
       </c>
       <c r="I124" s="29"/>
     </row>
-    <row r="125" ht="15" customHeight="1" spans="1:9">
-      <c r="A125" s="13"/>
+    <row r="125" ht="15" customHeight="1" spans="2:9">
       <c r="B125" s="28" t="s">
         <v>635</v>
       </c>
@@ -8911,8 +8788,7 @@
       </c>
       <c r="I125" s="29"/>
     </row>
-    <row r="126" ht="15" customHeight="1" spans="1:9">
-      <c r="A126" s="13"/>
+    <row r="126" ht="15" customHeight="1" spans="2:9">
       <c r="B126" s="28" t="s">
         <v>639</v>
       </c>
@@ -8928,8 +8804,7 @@
       </c>
       <c r="I126" s="29"/>
     </row>
-    <row r="127" ht="15" customHeight="1" spans="1:9">
-      <c r="A127" s="13"/>
+    <row r="127" ht="15" customHeight="1" spans="2:9">
       <c r="B127" s="28" t="s">
         <v>643</v>
       </c>
@@ -8945,8 +8820,7 @@
       </c>
       <c r="I127" s="29"/>
     </row>
-    <row r="128" ht="15" customHeight="1" spans="1:9">
-      <c r="A128" s="13"/>
+    <row r="128" ht="15" customHeight="1" spans="2:9">
       <c r="B128" s="28" t="s">
         <v>647</v>
       </c>
@@ -8962,8 +8836,7 @@
       </c>
       <c r="I128" s="29"/>
     </row>
-    <row r="129" ht="15" customHeight="1" spans="1:9">
-      <c r="A129" s="13"/>
+    <row r="129" ht="15" customHeight="1" spans="2:9">
       <c r="B129" s="28" t="s">
         <v>651</v>
       </c>
@@ -8979,8 +8852,7 @@
       </c>
       <c r="I129" s="29"/>
     </row>
-    <row r="130" ht="15" customHeight="1" spans="1:9">
-      <c r="A130" s="13"/>
+    <row r="130" ht="15" customHeight="1" spans="2:9">
       <c r="B130" s="28" t="s">
         <v>655</v>
       </c>
@@ -8996,8 +8868,7 @@
       </c>
       <c r="I130" s="29"/>
     </row>
-    <row r="131" ht="15" customHeight="1" spans="1:9">
-      <c r="A131" s="13"/>
+    <row r="131" ht="15" customHeight="1" spans="2:9">
       <c r="B131" s="28" t="s">
         <v>659</v>
       </c>
@@ -9013,8 +8884,7 @@
       </c>
       <c r="I131" s="29"/>
     </row>
-    <row r="132" ht="15" customHeight="1" spans="1:9">
-      <c r="A132" s="13"/>
+    <row r="132" ht="15" customHeight="1" spans="2:9">
       <c r="B132" s="28" t="s">
         <v>663</v>
       </c>
@@ -9030,8 +8900,7 @@
       </c>
       <c r="I132" s="29"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:9">
-      <c r="A133" s="13"/>
+    <row r="133" ht="15" customHeight="1" spans="2:9">
       <c r="B133" s="36" t="s">
         <v>667</v>
       </c>
@@ -9047,8 +8916,7 @@
       </c>
       <c r="I133" s="38"/>
     </row>
-    <row r="134" ht="15" customHeight="1" spans="1:9">
-      <c r="A134" s="13"/>
+    <row r="134" ht="15" customHeight="1" spans="2:9">
       <c r="B134" s="24" t="s">
         <v>671</v>
       </c>
@@ -9064,8 +8932,7 @@
       </c>
       <c r="I134" s="26"/>
     </row>
-    <row r="135" ht="15" customHeight="1" spans="1:9">
-      <c r="A135" s="13"/>
+    <row r="135" ht="15" customHeight="1" spans="2:9">
       <c r="B135" s="28" t="s">
         <v>673</v>
       </c>
@@ -9081,8 +8948,7 @@
       </c>
       <c r="I135" s="29"/>
     </row>
-    <row r="136" ht="15" customHeight="1" spans="1:9">
-      <c r="A136" s="13"/>
+    <row r="136" ht="15" customHeight="1" spans="2:9">
       <c r="B136" s="28" t="s">
         <v>675</v>
       </c>
@@ -9098,8 +8964,7 @@
       </c>
       <c r="I136" s="29"/>
     </row>
-    <row r="137" ht="15" customHeight="1" spans="1:9">
-      <c r="A137" s="13"/>
+    <row r="137" ht="15" customHeight="1" spans="2:9">
       <c r="B137" s="28" t="s">
         <v>677</v>
       </c>
@@ -9115,8 +8980,7 @@
       </c>
       <c r="I137" s="29"/>
     </row>
-    <row r="138" ht="15" customHeight="1" spans="1:9">
-      <c r="A138" s="13"/>
+    <row r="138" ht="15" customHeight="1" spans="2:9">
       <c r="B138" s="28" t="s">
         <v>679</v>
       </c>
@@ -9132,8 +8996,7 @@
       </c>
       <c r="I138" s="29"/>
     </row>
-    <row r="139" ht="15" customHeight="1" spans="1:9">
-      <c r="A139" s="13"/>
+    <row r="139" ht="15" customHeight="1" spans="2:9">
       <c r="B139" s="28" t="s">
         <v>681</v>
       </c>
@@ -9149,8 +9012,7 @@
       </c>
       <c r="I139" s="29"/>
     </row>
-    <row r="140" ht="15" customHeight="1" spans="1:9">
-      <c r="A140" s="13"/>
+    <row r="140" ht="15" customHeight="1" spans="2:9">
       <c r="B140" s="28" t="s">
         <v>683</v>
       </c>
@@ -9166,8 +9028,7 @@
       </c>
       <c r="I140" s="29"/>
     </row>
-    <row r="141" ht="15" customHeight="1" spans="1:9">
-      <c r="A141" s="13"/>
+    <row r="141" ht="15" customHeight="1" spans="2:9">
       <c r="B141" s="28" t="s">
         <v>685</v>
       </c>
@@ -9183,8 +9044,7 @@
       </c>
       <c r="I141" s="29"/>
     </row>
-    <row r="142" ht="15" customHeight="1" spans="1:9">
-      <c r="A142" s="13"/>
+    <row r="142" ht="15" customHeight="1" spans="2:9">
       <c r="B142" s="28" t="s">
         <v>687</v>
       </c>
@@ -9200,8 +9060,7 @@
       </c>
       <c r="I142" s="29"/>
     </row>
-    <row r="143" ht="15" customHeight="1" spans="1:9">
-      <c r="A143" s="13"/>
+    <row r="143" ht="15" customHeight="1" spans="2:9">
       <c r="B143" s="28" t="s">
         <v>689</v>
       </c>
@@ -9217,8 +9076,7 @@
       </c>
       <c r="I143" s="29"/>
     </row>
-    <row r="144" ht="15" customHeight="1" spans="1:9">
-      <c r="A144" s="13"/>
+    <row r="144" ht="15" customHeight="1" spans="2:9">
       <c r="B144" s="28" t="s">
         <v>691</v>
       </c>
@@ -16251,8 +16109,7 @@
       <c r="I655" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:A144"/>
+  <mergeCells count="2">
     <mergeCell ref="F2:F57"/>
     <mergeCell ref="K2:M9"/>
   </mergeCells>
@@ -16332,52 +16189,52 @@
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
     </row>
-    <row r="21" ht="14.25" spans="1:3">
+    <row r="21" ht="13.85" spans="1:3">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
     </row>
-    <row r="22" ht="14.25" spans="1:3">
+    <row r="22" ht="13.85" spans="1:3">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
     </row>
-    <row r="23" ht="14.25" spans="1:3">
+    <row r="23" ht="13.85" spans="1:3">
       <c r="A23" s="10"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
     </row>
-    <row r="24" ht="14.25" spans="1:3">
+    <row r="24" ht="13.85" spans="1:3">
       <c r="A24" s="10"/>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
     </row>
-    <row r="25" ht="14.25" spans="1:3">
+    <row r="25" ht="13.85" spans="1:3">
       <c r="A25" s="10"/>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
     </row>
-    <row r="26" ht="14.25" spans="1:3">
+    <row r="26" ht="13.85" spans="1:3">
       <c r="A26" s="10"/>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
     </row>
-    <row r="27" ht="14.25" spans="1:3">
+    <row r="27" ht="13.85" spans="1:3">
       <c r="A27" s="10"/>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
     </row>
-    <row r="28" ht="14.25" spans="1:3">
+    <row r="28" ht="13.85" spans="1:3">
       <c r="A28" s="10"/>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
     </row>
-    <row r="29" ht="14.25" spans="1:3">
+    <row r="29" ht="13.85" spans="1:3">
       <c r="A29" s="10"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
     </row>
-    <row r="30" ht="14.25" spans="1:3">
+    <row r="30" ht="13.85" spans="1:3">
       <c r="A30" s="10" t="s">
         <v>1279</v>
       </c>
@@ -16386,7 +16243,7 @@
       </c>
       <c r="C30" s="13"/>
     </row>
-    <row r="31" ht="14.25" spans="1:3">
+    <row r="31" ht="13.85" spans="1:3">
       <c r="A31" s="10" t="s">
         <v>1281</v>
       </c>
@@ -16397,7 +16254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" ht="14.25" spans="1:3">
+    <row r="32" ht="13.85" spans="1:3">
       <c r="A32" s="10" t="s">
         <v>1283</v>
       </c>
@@ -16408,7 +16265,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" ht="14.25" spans="1:3">
+    <row r="33" ht="13.85" spans="1:3">
       <c r="A33" s="10" t="s">
         <v>1285</v>
       </c>
@@ -16419,7 +16276,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" ht="14.25" spans="1:3">
+    <row r="34" ht="13.85" spans="1:3">
       <c r="A34" s="10" t="s">
         <v>1287</v>
       </c>
@@ -16430,7 +16287,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" ht="14.25" spans="1:3">
+    <row r="35" ht="13.85" spans="1:3">
       <c r="A35" s="10" t="s">
         <v>1289</v>
       </c>
@@ -16441,7 +16298,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" ht="14.25" spans="1:3">
+    <row r="36" ht="13.85" spans="1:3">
       <c r="A36" s="10" t="s">
         <v>1291</v>
       </c>
@@ -16452,7 +16309,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" ht="14.25" spans="1:3">
+    <row r="37" ht="13.85" spans="1:3">
       <c r="A37" s="10" t="s">
         <v>1293</v>
       </c>
@@ -16463,7 +16320,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="38" ht="14.25" spans="1:3">
+    <row r="38" ht="13.85" spans="1:3">
       <c r="A38" s="10"/>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
@@ -16477,42 +16334,42 @@
         <v>1296</v>
       </c>
     </row>
-    <row r="40" ht="14.25" spans="1:3">
+    <row r="40" ht="13.85" spans="1:3">
       <c r="A40" s="10"/>
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
     </row>
-    <row r="41" ht="14.25" spans="1:3">
+    <row r="41" ht="13.85" spans="1:3">
       <c r="A41" s="10"/>
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
     </row>
-    <row r="42" ht="14.25" spans="1:3">
+    <row r="42" ht="13.85" spans="1:3">
       <c r="A42" s="10"/>
       <c r="B42" s="11"/>
       <c r="C42" s="11"/>
     </row>
-    <row r="43" ht="14.25" spans="1:3">
+    <row r="43" ht="13.85" spans="1:3">
       <c r="A43" s="10"/>
       <c r="B43" s="11"/>
       <c r="C43" s="11"/>
     </row>
-    <row r="44" ht="14.25" spans="1:3">
+    <row r="44" ht="13.85" spans="1:3">
       <c r="A44" s="10"/>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
     </row>
-    <row r="45" ht="14.25" spans="1:3">
+    <row r="45" ht="13.85" spans="1:3">
       <c r="A45" s="10"/>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
     </row>
-    <row r="46" ht="14.25" spans="1:3">
+    <row r="46" ht="13.85" spans="1:3">
       <c r="A46" s="10"/>
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
     </row>
-    <row r="47" ht="14.25" spans="1:3">
+    <row r="47" ht="13.85" spans="1:3">
       <c r="A47" s="10"/>
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
@@ -16522,42 +16379,42 @@
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
     </row>
-    <row r="49" ht="14.25" spans="1:3">
+    <row r="49" ht="13.85" spans="1:3">
       <c r="A49" s="10"/>
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
     </row>
-    <row r="50" ht="14.25" spans="1:3">
+    <row r="50" ht="13.85" spans="1:3">
       <c r="A50" s="10"/>
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
     </row>
-    <row r="51" ht="14.25" spans="1:3">
+    <row r="51" ht="13.85" spans="1:3">
       <c r="A51" s="10"/>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
     </row>
-    <row r="52" ht="14.25" spans="1:3">
+    <row r="52" ht="13.85" spans="1:3">
       <c r="A52" s="10"/>
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
     </row>
-    <row r="53" ht="14.25" spans="1:3">
+    <row r="53" ht="13.85" spans="1:3">
       <c r="A53" s="10"/>
       <c r="B53" s="11"/>
       <c r="C53" s="11"/>
     </row>
-    <row r="54" ht="14.25" spans="1:3">
+    <row r="54" ht="13.85" spans="1:3">
       <c r="A54" s="10"/>
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
     </row>
-    <row r="55" ht="14.25" spans="1:3">
+    <row r="55" ht="13.85" spans="1:3">
       <c r="A55" s="10"/>
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
     </row>
-    <row r="56" ht="14.25" spans="1:3">
+    <row r="56" ht="13.85" spans="1:3">
       <c r="A56" s="10"/>
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
@@ -16567,40 +16424,40 @@
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
     </row>
-    <row r="58" ht="14.25" spans="1:3">
+    <row r="58" ht="13.85" spans="1:3">
       <c r="A58" s="10"/>
       <c r="B58" s="11"/>
       <c r="C58" s="11"/>
     </row>
-    <row r="59" ht="14.25" spans="1:3">
+    <row r="59" ht="13.85" spans="1:3">
       <c r="A59" s="10"/>
       <c r="B59" s="11"/>
       <c r="C59" s="11"/>
     </row>
-    <row r="68" ht="14.25" spans="1:3">
+    <row r="68" ht="13.85" spans="1:3">
       <c r="A68" s="10"/>
       <c r="B68" s="11"/>
       <c r="C68" s="11"/>
     </row>
-    <row r="69" ht="14.25" spans="1:3">
+    <row r="69" ht="13.85" spans="1:3">
       <c r="A69" s="10"/>
       <c r="B69" s="11"/>
       <c r="C69" s="11"/>
     </row>
-    <row r="70" ht="14.25" spans="1:1">
+    <row r="70" ht="13.85" spans="1:1">
       <c r="A70" s="10"/>
     </row>
-    <row r="71" ht="14.25" spans="1:3">
+    <row r="71" ht="13.85" spans="1:3">
       <c r="A71" s="10"/>
       <c r="B71" s="11"/>
       <c r="C71" s="11"/>
     </row>
-    <row r="72" ht="14.25" spans="1:3">
+    <row r="72" ht="13.85" spans="1:3">
       <c r="A72" s="10"/>
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
     </row>
-    <row r="73" ht="14.25" spans="1:3">
+    <row r="73" ht="13.85" spans="1:3">
       <c r="A73" s="10"/>
       <c r="B73" s="11"/>
       <c r="C73" s="11"/>
@@ -16610,82 +16467,82 @@
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
     </row>
-    <row r="75" ht="14.25" spans="1:3">
+    <row r="75" ht="13.85" spans="1:3">
       <c r="A75" s="10"/>
       <c r="B75" s="11"/>
       <c r="C75" s="11"/>
     </row>
-    <row r="76" ht="14.25" spans="1:3">
+    <row r="76" ht="13.85" spans="1:3">
       <c r="A76" s="10"/>
       <c r="B76" s="11"/>
       <c r="C76" s="11"/>
     </row>
-    <row r="77" ht="14.25" spans="1:3">
+    <row r="77" ht="13.85" spans="1:3">
       <c r="A77" s="10"/>
       <c r="B77" s="11"/>
       <c r="C77" s="11"/>
     </row>
-    <row r="78" ht="14.25" spans="1:3">
+    <row r="78" ht="13.85" spans="1:3">
       <c r="A78" s="10"/>
       <c r="B78" s="11"/>
       <c r="C78" s="11"/>
     </row>
-    <row r="79" ht="14.25" spans="1:3">
+    <row r="79" ht="13.85" spans="1:3">
       <c r="A79" s="10"/>
       <c r="B79" s="11"/>
       <c r="C79" s="11"/>
     </row>
-    <row r="80" ht="14.25" spans="1:3">
+    <row r="80" ht="13.85" spans="1:3">
       <c r="A80" s="10"/>
       <c r="B80" s="11"/>
       <c r="C80" s="11"/>
     </row>
-    <row r="81" ht="14.25" spans="1:3">
+    <row r="81" ht="13.85" spans="1:3">
       <c r="A81" s="10"/>
       <c r="B81" s="11"/>
       <c r="C81" s="11"/>
     </row>
-    <row r="82" ht="14.25" spans="1:3">
+    <row r="82" ht="13.85" spans="1:3">
       <c r="A82" s="10"/>
       <c r="B82" s="11"/>
       <c r="C82" s="11"/>
     </row>
-    <row r="83" ht="14.25" spans="1:3">
+    <row r="83" ht="13.85" spans="1:3">
       <c r="A83" s="10"/>
       <c r="B83" s="11"/>
       <c r="C83" s="11"/>
     </row>
-    <row r="84" ht="14.25" spans="1:3">
+    <row r="84" ht="13.85" spans="1:3">
       <c r="A84" s="10"/>
       <c r="B84" s="11"/>
       <c r="C84" s="11"/>
     </row>
-    <row r="85" ht="14.25" spans="1:3">
+    <row r="85" ht="13.85" spans="1:3">
       <c r="A85" s="10"/>
       <c r="B85" s="11"/>
       <c r="C85" s="11"/>
     </row>
-    <row r="86" ht="14.25" spans="1:3">
+    <row r="86" ht="13.85" spans="1:3">
       <c r="A86" s="10"/>
       <c r="B86" s="11"/>
       <c r="C86" s="11"/>
     </row>
-    <row r="87" ht="14.25" spans="1:3">
+    <row r="87" ht="13.85" spans="1:3">
       <c r="A87" s="10"/>
       <c r="B87" s="11"/>
       <c r="C87" s="11"/>
     </row>
-    <row r="88" ht="14.25" spans="1:3">
+    <row r="88" ht="13.85" spans="1:3">
       <c r="A88" s="10"/>
       <c r="B88" s="11"/>
       <c r="C88" s="11"/>
     </row>
-    <row r="89" ht="14.25" spans="1:3">
+    <row r="89" ht="13.85" spans="1:3">
       <c r="A89" s="10"/>
       <c r="B89" s="11"/>
       <c r="C89" s="11"/>
     </row>
-    <row r="90" ht="14.25" spans="1:3">
+    <row r="90" ht="13.85" spans="1:3">
       <c r="A90" s="10"/>
       <c r="B90" s="11"/>
       <c r="C90" s="11"/>

</xml_diff>